<commit_message>
Revert dynamic toggle text for different languages
</commit_message>
<xml_diff>
--- a/package/translations.xlsx
+++ b/package/translations.xlsx
@@ -417,12 +417,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="41" customWidth="1" min="1" max="1"/>
-    <col width="80" customWidth="1" min="2" max="2"/>
-    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="90" customWidth="1" min="2" max="2"/>
+    <col width="51" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
@@ -492,6 +492,116 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>title01</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>一般</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>常规</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>toggle01</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Enable Auto Place Fishing Items</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>釣りアイテムの自動配置を有効化</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>启用钓鱼物品自动放置</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>tooltip01</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Enable or disable sending tracked fishing catches to containers whose permission is set to shared.</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>追跡された釣果を、権限が「共有中」に設定されているコンテナへ送るかどうかを有効または無効にします。</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>启用或禁用将已追踪的钓鱼收获送入权限设为共享的容器。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>toggle02</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Enable Resident Require Bait</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>住人の餌要求を有効化</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>启用居民需要鱼饵</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>tooltip02</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Enable or disable requiring player bait for resident/follower catch delivery.</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>住人や仲間の釣果配達にプレイヤーの餌を必要とするかどうかを有効または無効にします。</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>启用或禁用居民或同伴收获送达时需要玩家鱼饵。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>